<commit_message>
dataset uploaded, group topic selected
</commit_message>
<xml_diff>
--- a/submissions/GroupFormation/STA380GroupForm.xlsx
+++ b/submissions/GroupFormation/STA380GroupForm.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="14440"/>
+    <workbookView windowHeight="14440"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>If left blank, you will be assigned a number.</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>Topic Number 1</t>
+  </si>
+  <si>
+    <t>Topic 8  (Advanced) Bootstrap Estimate</t>
   </si>
   <si>
     <t>Simulated distributions, if applicable:</t>
@@ -1277,7 +1280,7 @@
   <sheetFormatPr defaultColWidth="12.6339285714286" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="31.6339285714286" customWidth="1"/>
-    <col min="2" max="2" width="16.8303571428571" customWidth="1"/>
+    <col min="2" max="2" width="35.3660714285714" customWidth="1"/>
     <col min="3" max="3" width="15.25" customWidth="1"/>
     <col min="4" max="4" width="18.1339285714286" customWidth="1"/>
     <col min="5" max="5" width="16.3839285714286" customWidth="1"/>
@@ -1305,19 +1308,22 @@
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" customHeight="1" spans="1:1">
+    <row r="5" customHeight="1" spans="1:2">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="6" customHeight="1" spans="1:1">
       <c r="A6" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customHeight="1" spans="1:1">
       <c r="A7" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:1">
@@ -1328,17 +1334,17 @@
     </row>
     <row r="10" customHeight="1" spans="1:1">
       <c r="A10" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" customHeight="1" spans="1:1">
       <c r="A11" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customHeight="1" spans="1:1">
       <c r="A12" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" customHeight="1" spans="1:1">
@@ -1349,17 +1355,17 @@
     </row>
     <row r="15" customHeight="1" spans="1:1">
       <c r="A15" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customHeight="1" spans="1:1">
       <c r="A16" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="1:1">
       <c r="A17" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="1:1">
@@ -1368,124 +1374,124 @@
     <row r="20" customHeight="1" spans="1:6">
       <c r="A20" s="1"/>
       <c r="B20" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" customHeight="1" spans="1:6">
       <c r="A21" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21">
         <v>1009979347</v>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" customHeight="1" spans="1:6">
       <c r="A22" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D22">
         <v>1010541816</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" customHeight="1" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C23" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D23">
         <v>1010305028</v>
       </c>
       <c r="E23" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F23" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" customHeight="1" spans="1:6">
       <c r="A24" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D24">
         <v>1006895941</v>
       </c>
       <c r="E24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F24" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" customHeight="1" spans="1:1">
       <c r="A25" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" customHeight="1" spans="1:1">
       <c r="A27" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="1:1">
       <c r="A28" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" customHeight="1" spans="1:1">
       <c r="A29" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" customHeight="1" spans="1:1">
       <c r="A30" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>